<commit_message>
Update Excel artifact with new sheets and update pipeline
</commit_message>
<xml_diff>
--- a/E2E_Test_Report_TMS_2026-06-13T06-35-17.xlsx
+++ b/E2E_Test_Report_TMS_2026-06-13T06-35-17.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Passed Tests" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Failed Tests" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Execution Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Details" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passed Tests" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failed Tests" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Details" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home Page" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login &amp; Registration" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Portal" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doctor Portal" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Portal" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,90 +434,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Test Suite</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Overall Status</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Total Tests</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Pass Rate %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Duration (sec)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>End Time</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TMS E2E Functionality Tests</t>
+          <t>TMS Full E2E</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" t="n">
+        <v>42.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Testcase</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>✅ ALL PASSED</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>133</v>
-      </c>
-      <c r="D2" t="n">
-        <v>133</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>14.26</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-06-13 06:35:03</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-06-13 06:35:17</t>
+          <t>0.44s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.5s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0.49s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.22s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.65s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.86s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.8s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.89s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.39s</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Verify Admin Portal feature 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1.36s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -576,7 +752,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -597,7 +772,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -618,7 +792,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -639,7 +812,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -660,7 +832,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -681,7 +852,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -702,7 +872,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -723,7 +892,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -744,7 +912,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -765,7 +932,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -786,7 +952,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -807,7 +972,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -828,7 +992,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -849,7 +1012,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -870,7 +1032,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -891,7 +1052,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -912,7 +1072,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -933,7 +1092,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -954,7 +1112,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -975,7 +1132,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -996,7 +1152,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1017,7 +1172,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1038,7 +1192,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1059,7 +1212,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1080,7 +1232,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1101,7 +1252,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1122,7 +1272,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1143,7 +1292,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1164,7 +1312,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1185,7 +1332,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1206,7 +1352,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1227,7 +1372,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1248,7 +1392,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1269,7 +1412,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1290,7 +1432,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1311,7 +1452,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1332,7 +1472,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1353,7 +1492,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1374,7 +1512,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1395,7 +1532,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1416,7 +1552,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1437,7 +1572,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1458,7 +1592,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1479,7 +1612,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1500,7 +1632,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1521,7 +1652,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1542,7 +1672,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1563,7 +1692,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1584,7 +1712,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1605,7 +1732,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1626,7 +1752,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1647,7 +1772,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1668,7 +1792,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1689,7 +1812,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1710,7 +1832,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1731,7 +1852,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1752,7 +1872,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1773,7 +1892,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1794,7 +1912,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1815,7 +1932,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1836,7 +1952,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1857,7 +1972,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1878,7 +1992,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1899,7 +2012,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1920,7 +2032,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1941,7 +2052,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1962,7 +2072,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1983,7 +2092,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2004,7 +2112,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2025,7 +2132,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2046,7 +2152,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2067,7 +2172,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2088,7 +2192,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2109,7 +2212,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2130,7 +2232,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2151,7 +2252,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2172,7 +2272,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2193,7 +2292,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2214,7 +2312,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2235,7 +2332,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2256,7 +2352,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2277,7 +2372,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2298,7 +2392,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2319,7 +2412,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2340,7 +2432,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2361,7 +2452,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2382,7 +2472,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2403,7 +2492,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2424,7 +2512,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2445,7 +2532,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2466,7 +2552,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2487,7 +2572,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2508,7 +2592,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2529,7 +2612,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2550,7 +2632,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2571,7 +2652,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2592,7 +2672,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2613,7 +2692,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2634,7 +2712,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2655,7 +2732,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2676,7 +2752,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2697,7 +2772,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2718,7 +2792,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2739,7 +2812,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2760,7 +2832,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2781,7 +2852,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2802,7 +2872,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2823,7 +2892,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2844,7 +2912,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2865,7 +2932,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2886,7 +2952,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2907,7 +2972,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2928,7 +2992,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2949,7 +3012,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2970,7 +3032,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2991,7 +3052,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -3012,7 +3072,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -3033,7 +3092,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -3054,7 +3112,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -3075,7 +3132,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -3096,7 +3152,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -3117,7 +3172,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -3138,7 +3192,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -3159,7 +3212,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -3180,7 +3232,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -3201,7 +3252,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -3222,7 +3272,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -3243,7 +3292,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -3264,7 +3312,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -3285,7 +3332,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -3306,7 +3352,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -3327,7 +3372,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -3348,7 +3392,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3451,7 +3494,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3472,7 +3514,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3493,7 +3534,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3514,7 +3554,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3535,7 +3574,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3556,7 +3594,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3577,7 +3614,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3598,7 +3634,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3619,7 +3654,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -3640,7 +3674,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -3661,7 +3694,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3682,7 +3714,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -3703,7 +3734,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -3724,7 +3754,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3745,7 +3774,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -3766,7 +3794,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -3787,7 +3814,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3808,7 +3834,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3829,7 +3854,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3850,7 +3874,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3871,7 +3894,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3892,7 +3914,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3913,7 +3934,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3934,7 +3954,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3955,7 +3974,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3976,7 +3994,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3997,7 +4014,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4018,7 +4034,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4039,7 +4054,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4060,7 +4074,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4081,7 +4094,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4102,7 +4114,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4123,7 +4134,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4144,7 +4154,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -4165,7 +4174,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4186,7 +4194,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4207,7 +4214,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4228,7 +4234,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4249,7 +4254,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -4270,7 +4274,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -4291,7 +4294,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -4312,7 +4314,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -4333,7 +4334,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -4354,7 +4354,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -4375,7 +4374,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -4396,7 +4394,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4417,7 +4414,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4438,7 +4434,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4459,7 +4454,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4480,7 +4474,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4501,7 +4494,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4522,7 +4514,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4543,7 +4534,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4564,7 +4554,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4585,7 +4574,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4606,7 +4594,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4627,7 +4614,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4648,7 +4634,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4669,7 +4654,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4690,7 +4674,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4711,7 +4694,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4732,7 +4714,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4753,7 +4734,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4774,7 +4754,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4795,7 +4774,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4816,7 +4794,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4837,7 +4814,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4858,7 +4834,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4879,7 +4854,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4900,7 +4874,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4921,7 +4894,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4942,7 +4914,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4963,7 +4934,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4984,7 +4954,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5005,7 +4974,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5026,7 +4994,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5047,7 +5014,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -5068,7 +5034,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5089,7 +5054,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5110,7 +5074,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -5131,7 +5094,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5152,7 +5114,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5173,7 +5134,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5194,7 +5154,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5215,7 +5174,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5236,7 +5194,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5257,7 +5214,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5278,7 +5234,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5299,7 +5254,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5320,7 +5274,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -5341,7 +5294,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5362,7 +5314,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5383,7 +5334,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5404,7 +5354,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5425,7 +5374,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5446,7 +5394,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5467,7 +5414,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -5488,7 +5434,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5509,7 +5454,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5530,7 +5474,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -5551,7 +5494,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -5572,7 +5514,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -5593,7 +5534,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -5614,7 +5554,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -5635,7 +5574,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -5656,7 +5594,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5677,7 +5614,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5698,7 +5634,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -5719,7 +5654,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5740,7 +5674,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -5761,7 +5694,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -5782,7 +5714,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5803,7 +5734,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5824,7 +5754,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5845,7 +5774,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5866,7 +5794,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5887,7 +5814,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5908,7 +5834,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5929,7 +5854,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5950,7 +5874,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5971,7 +5894,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5992,7 +5914,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -6013,7 +5934,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -6034,7 +5954,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -6055,7 +5974,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -6076,7 +5994,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -6097,7 +6014,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -6118,7 +6034,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -6139,7 +6054,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -6160,7 +6074,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -6181,7 +6094,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -6202,7 +6114,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -6223,7 +6134,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6285,7 +6195,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -6306,7 +6215,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -6327,7 +6235,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -6348,7 +6255,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -6369,7 +6275,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -6390,7 +6295,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -6411,7 +6315,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -6432,7 +6335,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -6453,7 +6355,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -6474,7 +6375,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -6495,7 +6395,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -6516,7 +6415,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -6537,7 +6435,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -6558,7 +6455,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -6579,7 +6475,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -6600,7 +6495,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -6621,7 +6515,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -6642,7 +6535,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -6663,7 +6555,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -6684,7 +6575,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -6705,7 +6595,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -6726,7 +6615,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -6747,7 +6635,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -6768,7 +6655,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -6789,7 +6675,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -6810,7 +6695,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -6831,7 +6715,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -6852,7 +6735,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -6873,7 +6755,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -6894,7 +6775,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -6915,7 +6795,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -6936,7 +6815,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -6957,7 +6835,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -6978,7 +6855,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -6999,7 +6875,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -7020,7 +6895,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -7041,7 +6915,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -7062,7 +6935,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -7083,7 +6955,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -7104,7 +6975,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -7125,7 +6995,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -7146,7 +7015,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -7167,7 +7035,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -7188,7 +7055,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -7209,7 +7075,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -7230,7 +7095,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -7251,7 +7115,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -7272,7 +7135,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -7293,7 +7155,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -7314,7 +7175,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -7335,7 +7195,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -7356,7 +7215,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -7377,7 +7235,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -7398,7 +7255,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -7419,7 +7275,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -7440,7 +7295,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -7461,7 +7315,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -7482,7 +7335,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -7503,7 +7355,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -7524,7 +7375,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -7545,7 +7395,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -7566,7 +7415,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -7587,7 +7435,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -7608,7 +7455,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -7629,7 +7475,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -7650,7 +7495,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -7671,7 +7515,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -7692,7 +7535,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -7713,7 +7555,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -7734,7 +7575,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -7755,7 +7595,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -7776,7 +7615,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -7797,7 +7635,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -7818,7 +7655,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -7839,7 +7675,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -7860,7 +7695,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -7881,7 +7715,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -7902,7 +7735,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -7923,7 +7755,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -7944,7 +7775,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -7965,7 +7795,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -7986,7 +7815,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -8007,7 +7835,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -8028,7 +7855,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -8049,7 +7875,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -8070,7 +7895,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -8091,7 +7915,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -8112,7 +7935,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -8133,7 +7955,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -8154,7 +7975,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -8175,7 +7995,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -8196,7 +8015,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -8217,7 +8035,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -8238,7 +8055,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -8259,7 +8075,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -8280,7 +8095,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -8301,7 +8115,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -8322,7 +8135,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -8343,7 +8155,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -8364,7 +8175,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -8385,7 +8195,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -8406,7 +8215,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -8427,7 +8235,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -8448,7 +8255,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -8469,7 +8275,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -8490,7 +8295,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -8511,7 +8315,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -8532,7 +8335,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -8553,7 +8355,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -8574,7 +8375,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -8595,7 +8395,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -8616,7 +8415,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -8637,7 +8435,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -8658,7 +8455,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -8679,7 +8475,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -8700,7 +8495,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -8721,7 +8515,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -8742,7 +8535,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -8763,7 +8555,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -8784,7 +8575,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -8805,7 +8595,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -8826,7 +8615,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -8847,7 +8635,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -8868,7 +8655,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -8889,7 +8675,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -8910,7 +8695,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -8931,7 +8715,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -8952,7 +8735,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -8973,7 +8755,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -8994,7 +8775,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -9015,7 +8795,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -9036,7 +8815,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -9057,7 +8835,810 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Testcase</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.12s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.65s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.27s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.76s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.43s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.94s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.66s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.38s</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Verify Home Page feature 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.95s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Testcase</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.97s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.41s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.87s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.93s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1.24s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.64s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.33s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.76s</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Verify Login &amp; Registration feature 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1.36s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Testcase</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.41s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.16s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.17s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.41s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1.16s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1.47s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.81s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.41s</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Verify Patient Portal feature 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.46s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Testcase</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1.15s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.01s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.28s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.37s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.91s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.74s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.56s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1.05s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.81s</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Verify Doctor Portal feature 10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1.16s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>